<commit_message>
data: publish 2026-10-13 sampler-linked operations analysis
</commit_message>
<xml_diff>
--- a/data/export/2026-10-13-182路.xlsx
+++ b/data/export/2026-10-13-182路.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC6"/>
+  <dimension ref="A1:AC10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -665,7 +665,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>05:50</t>
+          <t>06:22</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -715,7 +715,7 @@
       <c r="AB2" s="2" t="inlineStr"/>
       <c r="AC2" s="2" t="inlineStr">
         <is>
-          <t>—/5</t>
+          <t>—/9</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>05:50</t>
+          <t>06:22</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -826,7 +826,7 @@
       <c r="AB3" s="2" t="inlineStr"/>
       <c r="AC3" s="2" t="inlineStr">
         <is>
-          <t>—/5</t>
+          <t>—/9</t>
         </is>
       </c>
     </row>
@@ -887,7 +887,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>05:50</t>
+          <t>06:22</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -937,7 +937,7 @@
       <c r="AB4" s="2" t="inlineStr"/>
       <c r="AC4" s="2" t="inlineStr">
         <is>
-          <t>—/5</t>
+          <t>—/9</t>
         </is>
       </c>
     </row>
@@ -945,22 +945,22 @@
       <c r="A5" s="2" t="inlineStr"/>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>沪A67983D</t>
+          <t>沪A67026D</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>06:35</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
           <t>金杨路金口路</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>06:35</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>川沙客运站</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -998,7 +998,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>05:50</t>
+          <t>06:22</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -1048,7 +1048,7 @@
       <c r="AB5" s="2" t="inlineStr"/>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>—/5</t>
+          <t>—/9</t>
         </is>
       </c>
     </row>
@@ -1056,7 +1056,7 @@
       <c r="A6" s="2" t="inlineStr"/>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>沪A13735A</t>
+          <t>沪A67983D</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -1066,7 +1066,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>06:55</t>
+          <t>06:35</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -1109,7 +1109,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>05:50</t>
+          <t>06:22</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -1123,7 +1123,7 @@
       <c r="T6" s="2" t="inlineStr"/>
       <c r="U6" s="2" t="inlineStr">
         <is>
-          <t>06:55</t>
+          <t>06:35</t>
         </is>
       </c>
       <c r="V6" s="2" t="inlineStr">
@@ -1159,7 +1159,451 @@
       <c r="AB6" s="2" t="inlineStr"/>
       <c r="AC6" s="2" t="inlineStr">
         <is>
-          <t>—/5</t>
+          <t>—/9</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr"/>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>沪A68870D</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>06:48</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr"/>
+      <c r="K7" s="2" t="inlineStr"/>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr"/>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>06:12</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>06:22</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q7" s="2" t="inlineStr"/>
+      <c r="R7" s="2" t="inlineStr"/>
+      <c r="S7" s="2" t="inlineStr"/>
+      <c r="T7" s="2" t="inlineStr"/>
+      <c r="U7" s="2" t="inlineStr">
+        <is>
+          <t>06:48</t>
+        </is>
+      </c>
+      <c r="V7" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W7" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X7" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y7" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z7" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA7" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB7" s="2" t="inlineStr"/>
+      <c r="AC7" s="2" t="inlineStr">
+        <is>
+          <t>—/9</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr"/>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>沪A13735A</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>06:55</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr"/>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr"/>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>05:50</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>06:22</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q8" s="2" t="inlineStr"/>
+      <c r="R8" s="2" t="inlineStr"/>
+      <c r="S8" s="2" t="inlineStr"/>
+      <c r="T8" s="2" t="inlineStr"/>
+      <c r="U8" s="2" t="inlineStr">
+        <is>
+          <t>06:55</t>
+        </is>
+      </c>
+      <c r="V8" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W8" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X8" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y8" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z8" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA8" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB8" s="2" t="inlineStr"/>
+      <c r="AC8" s="2" t="inlineStr">
+        <is>
+          <t>—/9</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr"/>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>沪A32899D</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr"/>
+      <c r="K9" s="2" t="inlineStr"/>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr"/>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>06:22</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>06:22</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q9" s="2" t="inlineStr"/>
+      <c r="R9" s="2" t="inlineStr"/>
+      <c r="S9" s="2" t="inlineStr"/>
+      <c r="T9" s="2" t="inlineStr"/>
+      <c r="U9" s="2" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="V9" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W9" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X9" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y9" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z9" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA9" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB9" s="2" t="inlineStr"/>
+      <c r="AC9" s="2" t="inlineStr">
+        <is>
+          <t>—/9</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr"/>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>沪A67353D</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>07:15</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr"/>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>06:22</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q10" s="2" t="inlineStr"/>
+      <c r="R10" s="2" t="inlineStr"/>
+      <c r="S10" s="2" t="inlineStr"/>
+      <c r="T10" s="2" t="inlineStr"/>
+      <c r="U10" s="2" t="inlineStr">
+        <is>
+          <t>07:15</t>
+        </is>
+      </c>
+      <c r="V10" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W10" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X10" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y10" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z10" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA10" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB10" s="2" t="inlineStr"/>
+      <c r="AC10" s="2" t="inlineStr">
+        <is>
+          <t>—/9</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: publish 2026-10-13 rolling operations analysis
</commit_message>
<xml_diff>
--- a/data/export/2026-10-13-182路.xlsx
+++ b/data/export/2026-10-13-182路.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC39"/>
+  <dimension ref="A1:AC42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -669,7 +669,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>10:22</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -708,22 +708,22 @@
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AA2" s="2" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AA2" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
-          <t>79.0</t>
+          <t>78.7</t>
         </is>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
-          <t>3/14</t>
+          <t>4/14</t>
         </is>
       </c>
     </row>
@@ -788,7 +788,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>10:22</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -842,7 +842,7 @@
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
-          <t>7/14</t>
+          <t>8/14</t>
         </is>
       </c>
     </row>
@@ -907,7 +907,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>10:22</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -946,22 +946,22 @@
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AA4" s="2" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AA4" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
-          <t>81.5</t>
+          <t>77.7</t>
         </is>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
-          <t>6/14</t>
+          <t>3/14</t>
         </is>
       </c>
     </row>
@@ -1026,7 +1026,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>10:22</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -1070,17 +1070,17 @@
       </c>
       <c r="AA5" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
-          <t>89.0</t>
+          <t>82.7</t>
         </is>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>12/14</t>
+          <t>10/14</t>
         </is>
       </c>
     </row>
@@ -1145,7 +1145,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>10:22</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -1199,7 +1199,7 @@
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
-          <t>11/14</t>
+          <t>14/14</t>
         </is>
       </c>
     </row>
@@ -1264,7 +1264,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>10:22</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1318,7 +1318,7 @@
       </c>
       <c r="AC7" s="2" t="inlineStr">
         <is>
-          <t>9/14</t>
+          <t>11/14</t>
         </is>
       </c>
     </row>
@@ -1383,7 +1383,7 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>10:22</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
@@ -1437,7 +1437,7 @@
       </c>
       <c r="AC8" s="2" t="inlineStr">
         <is>
-          <t>8/14</t>
+          <t>9/14</t>
         </is>
       </c>
     </row>
@@ -1556,7 +1556,7 @@
       </c>
       <c r="AC9" s="2" t="inlineStr">
         <is>
-          <t>3/14</t>
+          <t>5/14</t>
         </is>
       </c>
     </row>
@@ -1621,7 +1621,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>10:22</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
@@ -1675,7 +1675,7 @@
       </c>
       <c r="AC10" s="2" t="inlineStr">
         <is>
-          <t>3/14</t>
+          <t>5/14</t>
         </is>
       </c>
     </row>
@@ -1740,7 +1740,7 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>10:22</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
@@ -1794,7 +1794,7 @@
       </c>
       <c r="AC11" s="2" t="inlineStr">
         <is>
-          <t>9/14</t>
+          <t>11/14</t>
         </is>
       </c>
     </row>
@@ -1855,7 +1855,7 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>10:22</t>
+          <t>10:32</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
@@ -1904,7 +1904,7 @@
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
-          <t>76.0</t>
+          <t>77.0</t>
         </is>
       </c>
       <c r="AC12" s="2" t="inlineStr">
@@ -1974,7 +1974,7 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>10:22</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
@@ -2013,22 +2013,22 @@
       </c>
       <c r="Z13" s="2" t="inlineStr">
         <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AA13" s="2" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AA13" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
-          <t>79.0</t>
+          <t>78.7</t>
         </is>
       </c>
       <c r="AC13" s="2" t="inlineStr">
         <is>
-          <t>3/14</t>
+          <t>4/14</t>
         </is>
       </c>
     </row>
@@ -2093,7 +2093,7 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>10:22</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
@@ -2137,17 +2137,17 @@
       </c>
       <c r="AA14" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
-          <t>98.0</t>
+          <t>83.5</t>
         </is>
       </c>
       <c r="AC14" s="2" t="inlineStr">
         <is>
-          <t>14/14</t>
+          <t>13/14</t>
         </is>
       </c>
     </row>
@@ -2212,7 +2212,7 @@
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>10:22</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
@@ -2251,22 +2251,22 @@
       </c>
       <c r="Z15" s="2" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA15" s="2" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="AA15" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
-          <t>96.0</t>
+          <t>81.0</t>
         </is>
       </c>
       <c r="AC15" s="2" t="inlineStr">
         <is>
-          <t>13/14</t>
+          <t>7/14</t>
         </is>
       </c>
     </row>
@@ -2331,7 +2331,7 @@
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>10:22</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
@@ -2370,22 +2370,22 @@
       </c>
       <c r="Z16" s="2" t="inlineStr">
         <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AA16" s="2" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AA16" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
-          <t>81.5</t>
+          <t>77.7</t>
         </is>
       </c>
       <c r="AC16" s="2" t="inlineStr">
         <is>
-          <t>6/14</t>
+          <t>3/14</t>
         </is>
       </c>
     </row>
@@ -2450,7 +2450,7 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>10:22</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
@@ -2504,7 +2504,7 @@
       </c>
       <c r="AC17" s="2" t="inlineStr">
         <is>
-          <t>7/14</t>
+          <t>8/14</t>
         </is>
       </c>
     </row>
@@ -2569,7 +2569,7 @@
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>10:22</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
@@ -2613,17 +2613,17 @@
       </c>
       <c r="AA18" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
-          <t>89.0</t>
+          <t>82.7</t>
         </is>
       </c>
       <c r="AC18" s="2" t="inlineStr">
         <is>
-          <t>12/14</t>
+          <t>10/14</t>
         </is>
       </c>
     </row>
@@ -2688,7 +2688,7 @@
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>10:22</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
@@ -2742,7 +2742,7 @@
       </c>
       <c r="AC19" s="2" t="inlineStr">
         <is>
-          <t>11/14</t>
+          <t>14/14</t>
         </is>
       </c>
     </row>
@@ -2807,7 +2807,7 @@
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>10:22</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
@@ -2926,7 +2926,7 @@
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>10:22</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
@@ -2980,7 +2980,7 @@
       </c>
       <c r="AC21" s="2" t="inlineStr">
         <is>
-          <t>9/14</t>
+          <t>11/14</t>
         </is>
       </c>
     </row>
@@ -3045,7 +3045,7 @@
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>10:22</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
@@ -3099,7 +3099,7 @@
       </c>
       <c r="AC22" s="2" t="inlineStr">
         <is>
-          <t>8/14</t>
+          <t>9/14</t>
         </is>
       </c>
     </row>
@@ -3218,7 +3218,7 @@
       </c>
       <c r="AC23" s="2" t="inlineStr">
         <is>
-          <t>3/14</t>
+          <t>5/14</t>
         </is>
       </c>
     </row>
@@ -3283,7 +3283,7 @@
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>10:22</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
@@ -3337,7 +3337,7 @@
       </c>
       <c r="AC24" s="2" t="inlineStr">
         <is>
-          <t>3/14</t>
+          <t>5/14</t>
         </is>
       </c>
     </row>
@@ -3402,7 +3402,7 @@
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>10:22</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
@@ -3456,7 +3456,7 @@
       </c>
       <c r="AC25" s="2" t="inlineStr">
         <is>
-          <t>9/14</t>
+          <t>11/14</t>
         </is>
       </c>
     </row>
@@ -3494,12 +3494,12 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>10:38</t>
+          <t>10:39</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>76分钟</t>
+          <t>77分钟</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr"/>
@@ -3521,7 +3521,7 @@
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>10:22</t>
+          <t>10:32</t>
         </is>
       </c>
       <c r="P26" s="2" t="inlineStr">
@@ -3570,7 +3570,7 @@
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
-          <t>76.0</t>
+          <t>77.0</t>
         </is>
       </c>
       <c r="AC26" s="2" t="inlineStr">
@@ -3613,12 +3613,12 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>10:40</t>
+          <t>10:39</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>70分钟</t>
+          <t>69分钟</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr"/>
@@ -3640,7 +3640,7 @@
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>10:22</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="P27" s="2" t="inlineStr">
@@ -3679,22 +3679,22 @@
       </c>
       <c r="Z27" s="2" t="inlineStr">
         <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AA27" s="2" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AA27" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
-          <t>79.0</t>
+          <t>78.7</t>
         </is>
       </c>
       <c r="AC27" s="2" t="inlineStr">
         <is>
-          <t>3/14</t>
+          <t>4/14</t>
         </is>
       </c>
     </row>
@@ -3722,32 +3722,36 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>10:44</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>69分钟</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr"/>
       <c r="K28" s="2" t="inlineStr"/>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M28" s="2" t="inlineStr"/>
+          <t>SHMAAS终点ETA近站估算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
           <t>07:02</t>
@@ -3755,7 +3759,7 @@
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>10:22</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="P28" s="2" t="inlineStr">
@@ -3779,17 +3783,17 @@
       </c>
       <c r="W28" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X28" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y28" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z28" s="2" t="inlineStr">
@@ -3799,17 +3803,17 @@
       </c>
       <c r="AA28" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
-          <t>98.0</t>
+          <t>83.5</t>
         </is>
       </c>
       <c r="AC28" s="2" t="inlineStr">
         <is>
-          <t>14/14</t>
+          <t>13/14</t>
         </is>
       </c>
     </row>
@@ -3837,32 +3841,36 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>10:56</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>66分钟</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr"/>
       <c r="K29" s="2" t="inlineStr"/>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M29" s="2" t="inlineStr"/>
+          <t>SHMAAS终点ETA近站估算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
           <t>07:22</t>
@@ -3870,7 +3878,7 @@
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>10:22</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="P29" s="2" t="inlineStr">
@@ -3894,37 +3902,37 @@
       </c>
       <c r="W29" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X29" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y29" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z29" s="2" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA29" s="2" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="AA29" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
-          <t>96.0</t>
+          <t>81.0</t>
         </is>
       </c>
       <c r="AC29" s="2" t="inlineStr">
         <is>
-          <t>13/14</t>
+          <t>7/14</t>
         </is>
       </c>
     </row>
@@ -3952,32 +3960,36 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>70分钟</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr"/>
       <c r="K30" s="2" t="inlineStr"/>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M30" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N30" s="2" t="inlineStr">
         <is>
           <t>05:50</t>
@@ -3985,7 +3997,7 @@
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>10:22</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="P30" s="2" t="inlineStr">
@@ -4009,37 +4021,37 @@
       </c>
       <c r="W30" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X30" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y30" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z30" s="2" t="inlineStr">
         <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AA30" s="2" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AA30" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
-          <t>81.5</t>
+          <t>77.7</t>
         </is>
       </c>
       <c r="AC30" s="2" t="inlineStr">
         <is>
-          <t>6/14</t>
+          <t>3/14</t>
         </is>
       </c>
     </row>
@@ -4100,7 +4112,7 @@
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>10:22</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="P31" s="2" t="inlineStr">
@@ -4154,7 +4166,7 @@
       </c>
       <c r="AC31" s="2" t="inlineStr">
         <is>
-          <t>7/14</t>
+          <t>8/14</t>
         </is>
       </c>
     </row>
@@ -4182,32 +4194,36 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>11:25</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>70分钟</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr"/>
       <c r="K32" s="2" t="inlineStr"/>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M32" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N32" s="2" t="inlineStr">
         <is>
           <t>05:50</t>
@@ -4215,7 +4231,7 @@
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>10:22</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="P32" s="2" t="inlineStr">
@@ -4239,17 +4255,17 @@
       </c>
       <c r="W32" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X32" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y32" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z32" s="2" t="inlineStr">
@@ -4259,17 +4275,17 @@
       </c>
       <c r="AA32" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
-          <t>89.0</t>
+          <t>82.7</t>
         </is>
       </c>
       <c r="AC32" s="2" t="inlineStr">
         <is>
-          <t>12/14</t>
+          <t>10/14</t>
         </is>
       </c>
     </row>
@@ -4330,7 +4346,7 @@
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>10:22</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="P33" s="2" t="inlineStr">
@@ -4384,7 +4400,7 @@
       </c>
       <c r="AC33" s="2" t="inlineStr">
         <is>
-          <t>11/14</t>
+          <t>14/14</t>
         </is>
       </c>
     </row>
@@ -4445,7 +4461,7 @@
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>10:22</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="P34" s="2" t="inlineStr">
@@ -4560,7 +4576,7 @@
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>10:22</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="P35" s="2" t="inlineStr">
@@ -4614,7 +4630,7 @@
       </c>
       <c r="AC35" s="2" t="inlineStr">
         <is>
-          <t>9/14</t>
+          <t>11/14</t>
         </is>
       </c>
     </row>
@@ -4675,7 +4691,7 @@
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>10:22</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="P36" s="2" t="inlineStr">
@@ -4729,7 +4745,7 @@
       </c>
       <c r="AC36" s="2" t="inlineStr">
         <is>
-          <t>8/14</t>
+          <t>9/14</t>
         </is>
       </c>
     </row>
@@ -4790,7 +4806,7 @@
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>10:22</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="P37" s="2" t="inlineStr">
@@ -4844,7 +4860,7 @@
       </c>
       <c r="AC37" s="2" t="inlineStr">
         <is>
-          <t>3/14</t>
+          <t>5/14</t>
         </is>
       </c>
     </row>
@@ -4905,7 +4921,7 @@
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>10:22</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="P38" s="2" t="inlineStr">
@@ -4959,7 +4975,7 @@
       </c>
       <c r="AC38" s="2" t="inlineStr">
         <is>
-          <t>9/14</t>
+          <t>11/14</t>
         </is>
       </c>
     </row>
@@ -4967,22 +4983,22 @@
       <c r="A39" s="2" t="inlineStr"/>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>沪A35717D</t>
+          <t>沪A32298D</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>11:20</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
           <t>川沙客运站</t>
-        </is>
-      </c>
-      <c r="D39" s="2" t="inlineStr">
-        <is>
-          <t>11:30</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr">
-        <is>
-          <t>金杨路金口路</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -5015,12 +5031,12 @@
       <c r="M39" s="2" t="inlineStr"/>
       <c r="N39" s="2" t="inlineStr">
         <is>
-          <t>07:02</t>
+          <t>05:50</t>
         </is>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
-          <t>10:22</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="P39" s="2" t="inlineStr">
@@ -5034,47 +5050,392 @@
       <c r="T39" s="2" t="inlineStr"/>
       <c r="U39" s="2" t="inlineStr">
         <is>
+          <t>11:20</t>
+        </is>
+      </c>
+      <c r="V39" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W39" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X39" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y39" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z39" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AA39" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AB39" s="2" t="inlineStr">
+        <is>
+          <t>78.7</t>
+        </is>
+      </c>
+      <c r="AC39" s="2" t="inlineStr">
+        <is>
+          <t>4/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr"/>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>沪A35717D</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
           <t>11:30</t>
         </is>
       </c>
-      <c r="V39" s="2" t="inlineStr">
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr"/>
+      <c r="K40" s="2" t="inlineStr"/>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M40" s="2" t="inlineStr"/>
+      <c r="N40" s="2" t="inlineStr">
+        <is>
+          <t>07:02</t>
+        </is>
+      </c>
+      <c r="O40" s="2" t="inlineStr">
+        <is>
+          <t>10:51</t>
+        </is>
+      </c>
+      <c r="P40" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q40" s="2" t="inlineStr"/>
+      <c r="R40" s="2" t="inlineStr"/>
+      <c r="S40" s="2" t="inlineStr"/>
+      <c r="T40" s="2" t="inlineStr"/>
+      <c r="U40" s="2" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="V40" s="2" t="inlineStr">
         <is>
           <t>计划发车</t>
         </is>
       </c>
-      <c r="W39" s="2" t="inlineStr">
+      <c r="W40" s="2" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="X39" s="2" t="inlineStr">
+      <c r="X40" s="2" t="inlineStr">
         <is>
           <t>待确认</t>
         </is>
       </c>
-      <c r="Y39" s="2" t="inlineStr">
+      <c r="Y40" s="2" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="Z39" s="2" t="inlineStr">
+      <c r="Z40" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AA39" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AB39" s="2" t="inlineStr">
-        <is>
-          <t>98.0</t>
-        </is>
-      </c>
-      <c r="AC39" s="2" t="inlineStr">
-        <is>
-          <t>14/14</t>
+      <c r="AA40" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AB40" s="2" t="inlineStr">
+        <is>
+          <t>83.5</t>
+        </is>
+      </c>
+      <c r="AC40" s="2" t="inlineStr">
+        <is>
+          <t>13/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr"/>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>沪A68397D</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>11:40</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr"/>
+      <c r="K41" s="2" t="inlineStr"/>
+      <c r="L41" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M41" s="2" t="inlineStr"/>
+      <c r="N41" s="2" t="inlineStr">
+        <is>
+          <t>05:50</t>
+        </is>
+      </c>
+      <c r="O41" s="2" t="inlineStr">
+        <is>
+          <t>10:51</t>
+        </is>
+      </c>
+      <c r="P41" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q41" s="2" t="inlineStr"/>
+      <c r="R41" s="2" t="inlineStr"/>
+      <c r="S41" s="2" t="inlineStr"/>
+      <c r="T41" s="2" t="inlineStr"/>
+      <c r="U41" s="2" t="inlineStr">
+        <is>
+          <t>11:40</t>
+        </is>
+      </c>
+      <c r="V41" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W41" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X41" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y41" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z41" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AA41" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AB41" s="2" t="inlineStr">
+        <is>
+          <t>77.7</t>
+        </is>
+      </c>
+      <c r="AC41" s="2" t="inlineStr">
+        <is>
+          <t>3/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr"/>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>沪A02126A</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>11:55</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr"/>
+      <c r="K42" s="2" t="inlineStr"/>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M42" s="2" t="inlineStr"/>
+      <c r="N42" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="O42" s="2" t="inlineStr">
+        <is>
+          <t>10:51</t>
+        </is>
+      </c>
+      <c r="P42" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q42" s="2" t="inlineStr"/>
+      <c r="R42" s="2" t="inlineStr"/>
+      <c r="S42" s="2" t="inlineStr"/>
+      <c r="T42" s="2" t="inlineStr"/>
+      <c r="U42" s="2" t="inlineStr">
+        <is>
+          <t>11:55</t>
+        </is>
+      </c>
+      <c r="V42" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W42" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X42" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y42" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z42" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA42" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AB42" s="2" t="inlineStr">
+        <is>
+          <t>81.0</t>
+        </is>
+      </c>
+      <c r="AC42" s="2" t="inlineStr">
+        <is>
+          <t>7/14</t>
         </is>
       </c>
     </row>

</xml_diff>